<commit_message>
TKB.xlsx: wider BUỔI and TIẾT columns
The two label columns were sized to the longest text only ("CHIỀU",
"TIẾT"), which looked cramped in bold 14 pt. They now get LABEL_PAD = 4
extra units (BUỔI 8.1 -> 12.1, TIẾT 6.9 -> 10.9 with the school's style).
Layout only: result codes are unchanged (fake school A77F-F330-8C78).
Output templates regenerated; the layout test checks the new widths.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B1DqxLw2MywB8g5N8E14F5
</commit_message>
<xml_diff>
--- a/data/Output_Template_TKB_V8.xlsx
+++ b/data/Output_Template_TKB_V8.xlsx
@@ -465,8 +465,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.5" customWidth="1" min="1" max="1"/>
-    <col width="8.1" customWidth="1" min="2" max="2"/>
-    <col width="6.9" customWidth="1" min="3" max="3"/>
+    <col width="12.1" customWidth="1" min="2" max="2"/>
+    <col width="10.9" customWidth="1" min="3" max="3"/>
     <col width="21.5" customWidth="1" min="4" max="4"/>
     <col width="21.5" customWidth="1" min="5" max="5"/>
     <col width="21.5" customWidth="1" min="6" max="6"/>
@@ -2370,8 +2370,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.5" customWidth="1" min="1" max="1"/>
-    <col width="8.1" customWidth="1" min="2" max="2"/>
-    <col width="6.9" customWidth="1" min="3" max="3"/>
+    <col width="12.1" customWidth="1" min="2" max="2"/>
+    <col width="10.9" customWidth="1" min="3" max="3"/>
     <col width="21.5" customWidth="1" min="4" max="4"/>
     <col width="21.5" customWidth="1" min="5" max="5"/>
     <col width="21.5" customWidth="1" min="6" max="6"/>
@@ -4275,8 +4275,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.5" customWidth="1" min="1" max="1"/>
-    <col width="8.1" customWidth="1" min="2" max="2"/>
-    <col width="6.9" customWidth="1" min="3" max="3"/>
+    <col width="12.1" customWidth="1" min="2" max="2"/>
+    <col width="10.9" customWidth="1" min="3" max="3"/>
     <col width="21.5" customWidth="1" min="4" max="4"/>
     <col width="21.5" customWidth="1" min="5" max="5"/>
     <col width="21.5" customWidth="1" min="6" max="6"/>
@@ -6180,8 +6180,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.5" customWidth="1" min="1" max="1"/>
-    <col width="8.1" customWidth="1" min="2" max="2"/>
-    <col width="6.9" customWidth="1" min="3" max="3"/>
+    <col width="12.1" customWidth="1" min="2" max="2"/>
+    <col width="10.9" customWidth="1" min="3" max="3"/>
     <col width="21.5" customWidth="1" min="4" max="4"/>
     <col width="21.5" customWidth="1" min="5" max="5"/>
     <col width="21.5" customWidth="1" min="6" max="6"/>
@@ -8085,8 +8085,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.5" customWidth="1" min="1" max="1"/>
-    <col width="8.1" customWidth="1" min="2" max="2"/>
-    <col width="6.9" customWidth="1" min="3" max="3"/>
+    <col width="12.1" customWidth="1" min="2" max="2"/>
+    <col width="10.9" customWidth="1" min="3" max="3"/>
     <col width="21.5" customWidth="1" min="4" max="4"/>
     <col width="21.5" customWidth="1" min="5" max="5"/>
     <col width="21.5" customWidth="1" min="6" max="6"/>

</xml_diff>

<commit_message>
Output templates and fake-school results for the 1200 default
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B1DqxLw2MywB8g5N8E14F5
</commit_message>
<xml_diff>
--- a/data/Output_Template_TKB_V8.xlsx
+++ b/data/Output_Template_TKB_V8.xlsx
@@ -569,25 +569,25 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>TNXH
-Giáo viên BM 1</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>Tiếng Anh
 Giáo viên TA 1</t>
         </is>
       </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
+Giáo viên CN 1</t>
+        </is>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên BM 1</t>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Kỹ năng sống
+          <t>TNXH
 Giáo viên BM 1</t>
         </is>
       </c>
@@ -649,14 +649,14 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 1</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
           <t>Tiếng Anh
 Giáo viên TA 1</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
+Giáo viên BM 1</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -684,8 +684,8 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
+          <t>Thể dục
+Giáo viên TD 3</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>TNXH
+          <t>Kỹ năng sống
 Giáo viên BM 1</t>
         </is>
       </c>
@@ -756,14 +756,14 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 3</t>
+          <t>TNXH
+Giáo viên BM 1</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 2</t>
         </is>
       </c>
@@ -897,8 +897,8 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 2</t>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 2</t>
         </is>
       </c>
@@ -971,8 +971,8 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
+          <t>Tiếng Việt
+Giáo viên CN 2</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>TNXH
+          <t>Kỹ năng sống
 Giáo viên BM 1</t>
         </is>
       </c>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Kỹ năng sống
+          <t>TNXH
 Giáo viên BM 1</t>
         </is>
       </c>
@@ -1189,8 +1189,8 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 1</t>
+          <t>Tiếng Việt
+Giáo viên CN 3</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1238,8 +1238,8 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 3</t>
+          <t>Tiếng Anh
+Giáo viên TA 1</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1263,14 +1263,14 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 3</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 1</t>
+          <t>Thể dục
+Giáo viên TD 3</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1304,8 +1304,8 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 3</t>
+          <t>Tiếng Anh
+Giáo viên TA 1</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1340,20 +1340,20 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
 Giáo viên CN 3</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Đạo đức
 Giáo viên CN 3</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Kỹ năng sống
-Giáo viên BM 1</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1376,22 +1376,22 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
+          <t>Thể dục
+Giáo viên TD 3</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Đạo đức
-Giáo viên CN 3</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>HĐTN
 Giáo viên CN 3</t>
         </is>
       </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Kỹ năng sống
+Giáo viên BM 1</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
           <t>TNXH
@@ -1468,7 +1468,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 4</t>
         </is>
       </c>
@@ -1499,26 +1499,26 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>TNXH
+Giáo viên BM 1</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
 Giáo viên CN 4</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 4</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 4</t>
-        </is>
-      </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
+          <t>Thể dục
+Giáo viên TD 1</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1536,14 +1536,14 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
+          <t>Kỹ năng sống
+Giáo viên BM 1</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
           <t>Tiếng Việt
 Giáo viên CN 4</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1573,20 +1573,20 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 4</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 4</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>TNXH
-Giáo viên BM 1</t>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Đạo đức
+          <t>Tiếng Việt
 Giáo viên CN 4</t>
         </is>
       </c>
@@ -1650,8 +1650,8 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
+          <t>Tiếng Việt
+Giáo viên CN 4</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1686,8 +1686,8 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Kỹ năng sống
-Giáo viên BM 1</t>
+          <t>Đạo đức
+Giáo viên CN 4</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -1698,16 +1698,16 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
+          <t>Thể dục
+Giáo viên TD 1</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
           <t>HĐTN
 Giáo viên CN 4</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
-        </is>
-      </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
           <t>Nghỉ</t>
@@ -1796,7 +1796,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 5</t>
         </is>
       </c>
@@ -1815,8 +1815,8 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>TNXH
-Giáo viên BM 2</t>
+          <t>Tiếng Anh
+Giáo viên TA 1</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -1858,8 +1858,8 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 5</t>
         </is>
       </c>
@@ -1924,8 +1924,8 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 1</t>
+          <t>Thể dục
+Giáo viên TD 1</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -1936,8 +1936,8 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 1</t>
+          <t>Thể dục
+Giáo viên TD 1</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -1960,8 +1960,8 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
+          <t>Tiếng Anh
+Giáo viên TA 1</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -1972,8 +1972,8 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
+          <t>Kỹ năng sống
+Giáo viên BM 1</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -1996,8 +1996,8 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2008,8 +2008,8 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Kỹ năng sống
-Giáo viên BM 1</t>
+          <t>TNXH
+Giáo viên BM 2</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -2119,20 +2119,20 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>TNXH
+Giáo viên BM 2</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Kỹ năng sống
+Giáo viên BM 2</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
 Giáo viên CN 6</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 6</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -2156,8 +2156,8 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 6</t>
+          <t>Tiếng Anh
+Giáo viên TA 1</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -2193,26 +2193,26 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 6</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Kỹ năng sống
+          <t>Tiếng Việt
+Giáo viên CN 6</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>TNXH
 Giáo viên BM 2</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 6</t>
-        </is>
-      </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 1</t>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2234,8 +2234,8 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
+          <t>Tiếng Việt
+Giáo viên CN 6</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -2252,8 +2252,8 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>TNXH
-Giáo viên BM 2</t>
+          <t>Tiếng Anh
+Giáo viên TA 1</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -2270,8 +2270,8 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 1</t>
+          <t>Tiếng Việt
+Giáo viên CN 6</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -2306,20 +2306,20 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>TNXH
-Giáo viên BM 2</t>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Thể dục
+Giáo viên TD 1</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>Đạo đức
 Giáo viên CN 6</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 7</t>
         </is>
       </c>
@@ -2517,14 +2517,14 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 7</t>
+          <t>TNXH
+Giáo viên BM 2</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
+          <t>Thể dục
+Giáo viên TD 1</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -2554,8 +2554,8 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
+          <t>Toán
+Giáo viên CN 7</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -2589,20 +2589,20 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>Toán tăng cường
 Giáo viên BM 2</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Đạo đức
-Giáo viên CN 7</t>
-        </is>
-      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Toán tăng cường
-Giáo viên BM 2</t>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>TNXH
+          <t>Toán tăng cường
 Giáo viên BM 2</t>
         </is>
       </c>
@@ -2661,28 +2661,28 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
+          <t>Kỹ năng sống
+Giáo viên BM 2</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Đạo đức
+Giáo viên CN 7</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>HĐTN
+Giáo viên CN 7</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>TNXH
 Giáo viên BM 2</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Kỹ năng sống
-Giáo viên BM 2</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>HĐTN
-Giáo viên CN 7</t>
-        </is>
-      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Nghỉ</t>
@@ -2753,19 +2753,19 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 8</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 8</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 8</t>
         </is>
       </c>
@@ -2790,14 +2790,14 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
+          <t>Thể dục
+Giáo viên TD 1</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>Tiếng Việt
 Giáo viên CN 8</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Kỹ năng sống
-Giáo viên BM 2</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -2821,25 +2821,25 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>Kỹ năng sống
+Giáo viên BM 2</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
+Giáo viên CN 8</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>TNXH
 Giáo viên BM 2</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>TNXH
-Giáo viên BM 2</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 8</t>
-        </is>
-      </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 8</t>
         </is>
       </c>
@@ -2864,20 +2864,20 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 8</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 8</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
+          <t>Tiếng Anh
+Giáo viên TA 1</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -2905,20 +2905,20 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
+          <t>TV tăng cường
+Giáo viên CN 8</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>Toán tăng cường
 Giáo viên BM 2</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>TV tăng cường
-Giáo viên CN 8</t>
-        </is>
-      </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 1</t>
+          <t>Thể dục
+Giáo viên TD 1</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -2941,14 +2941,14 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
           <t>TV tăng cường
 Giáo viên CN 8</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -2977,16 +2977,16 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
+          <t>TNXH
+Giáo viên BM 2</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>HĐTN
 Giáo viên CN 8</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
-        </is>
-      </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Mỹ thuật
@@ -3069,7 +3069,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 9</t>
         </is>
       </c>
@@ -3094,20 +3094,20 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 9</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
+          <t>Tiếng Việt
+Giáo viên CN 9</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 9</t>
+          <t>Thể dục
+Giáo viên TD 1</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -3131,8 +3131,8 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 1</t>
+          <t>Tiếng Việt
+Giáo viên CN 9</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -3143,8 +3143,8 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Kỹ năng sống
-Giáo viên BM 2</t>
+          <t>Tiếng Việt
+Giáo viên CN 9</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -3168,19 +3168,19 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
+          <t>Toán
+Giáo viên CN 9</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
           <t>TNXH
 Giáo viên BM 2</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 9</t>
-        </is>
-      </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 9</t>
         </is>
       </c>
@@ -3209,20 +3209,20 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 9</t>
+          <t>Toán tăng cường
+Giáo viên BM 2</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Thể dục
+Giáo viên TD 1</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Tiếng Anh
 Giáo viên TA 1</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -3245,8 +3245,8 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 9</t>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -3257,7 +3257,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Toán tăng cường
+          <t>Kỹ năng sống
 Giáo viên BM 2</t>
         </is>
       </c>
@@ -3281,22 +3281,22 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
+          <t>Tiếng Anh
+Giáo viên TA 1</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
           <t>Đạo đức
 Giáo viên CN 9</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
-        </is>
-      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
           <t>HĐTN
@@ -3373,7 +3373,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 10</t>
         </is>
       </c>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 10</t>
         </is>
       </c>
@@ -3410,8 +3410,8 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>TNXH
-Giáo viên BM 3</t>
+          <t>Tiếng Việt
+Giáo viên CN 10</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -3447,8 +3447,8 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 10</t>
+          <t>Thể dục
+Giáo viên TD 1</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 10</t>
         </is>
       </c>
@@ -3484,7 +3484,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 10</t>
         </is>
       </c>
@@ -3519,26 +3519,26 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Toán tăng cường
-Giáo viên BM 3</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Toán tăng cường
-Giáo viên BM 3</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
           <t>TV tăng cường
 Giáo viên CN 10</t>
         </is>
       </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Anh
+Giáo viên TA 1</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Đạo đức
+Giáo viên CN 10</t>
+        </is>
+      </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
+          <t>Kỹ năng sống
+Giáo viên BM 2</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -3555,20 +3555,20 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
           <t>TV tăng cường
 Giáo viên CN 10</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Toán tăng cường
+Giáo viên BM 3</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Toán tăng cường
+Giáo viên BM 3</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -3591,26 +3591,26 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 1</t>
+          <t>TNXH
+Giáo viên BM 3</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Đạo đức
-Giáo viên CN 10</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>HĐTN
 Giáo viên CN 10</t>
         </is>
       </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
+        </is>
+      </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Kỹ năng sống
-Giáo viên BM 2</t>
+          <t>Thể dục
+Giáo viên TD 1</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 11</t>
         </is>
       </c>
@@ -3763,8 +3763,8 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 1</t>
+          <t>Toán
+Giáo viên CN 11</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 11</t>
         </is>
       </c>
@@ -3800,8 +3800,8 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Toán
-Giáo viên CN 11</t>
+          <t>Tiếng Anh
+Giáo viên TA 1</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -3829,20 +3829,20 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Toán tăng cường
+Giáo viên BM 3</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>TV tăng cường
 Giáo viên CN 11</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -3865,26 +3865,26 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Toán tăng cường
+          <t>TNXH
 Giáo viên BM 3</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Thể dục
+Giáo viên TD 1</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>TV tăng cường
 Giáo viên CN 11</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
-        </is>
-      </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Đạo đức
-Giáo viên CN 11</t>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -3901,26 +3901,26 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
+          <t>Thể dục
+Giáo viên TD 1</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>HĐTN
+Giáo viên CN 11</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
           <t>TNXH
 Giáo viên BM 3</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>TNXH
-Giáo viên BM 3</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>HĐTN
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Đạo đức
 Giáo viên CN 11</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 12</t>
         </is>
       </c>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>TNXH
+          <t>Kỹ năng sống
 Giáo viên BM 3</t>
         </is>
       </c>
@@ -4098,7 +4098,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 12</t>
         </is>
       </c>
@@ -4110,8 +4110,8 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
+          <t>TNXH
+Giáo viên BM 3</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -4139,20 +4139,20 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
+          <t>Toán tăng cường
+Giáo viên BM 3</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
           <t>TV tăng cường
 Giáo viên CN 12</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>Thể dục
-Giáo viên TD 1</t>
-        </is>
-      </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Kỹ năng sống
-Giáo viên BM 3</t>
+          <t>Đạo đức
+Giáo viên CN 12</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -4175,20 +4175,20 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
+          <t>Thể dục
+Giáo viên TD 1</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
           <t>TV tăng cường
 Giáo viên CN 12</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
-        </is>
-      </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Toán tăng cường
-Giáo viên BM 3</t>
+          <t>Thể dục
+Giáo viên TD 1</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -4223,8 +4223,8 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Đạo đức
-Giáo viên CN 12</t>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -4354,7 +4354,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 13</t>
         </is>
       </c>
@@ -4379,8 +4379,8 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Toán
-Giáo viên CN 13</t>
+          <t>Thể dục
+Giáo viên TD 2</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -4422,25 +4422,25 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>Tiếng Việt
+Giáo viên CN 13</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Toán
+Giáo viên CN 13</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
+Giáo viên CN 13</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>TV tăng cường
-Giáo viên CN 13</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 13</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 13</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
 Giáo viên CN 13</t>
         </is>
       </c>
@@ -4453,14 +4453,14 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
+          <t>Toán
+Giáo viên CN 13</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 2</t>
+          <t>Công nghệ
+Giáo viên BM 3</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4506,8 +4506,8 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 2</t>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -4536,8 +4536,8 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Công nghệ
-Giáo viên BM 3</t>
+          <t>Tiếng Anh
+Giáo viên TA 2</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 14</t>
         </is>
       </c>
@@ -4689,8 +4689,8 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Toán
-Giáo viên CN 14</t>
+          <t>Tiếng Anh
+Giáo viên TA 2</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -4726,20 +4726,20 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>Toán
+Giáo viên CN 14</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
+Giáo viên CN 14</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>Tiếng Anh
 Giáo viên TA 2</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 14</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 14</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -4775,8 +4775,8 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Công nghệ
-Giáo viên BM 3</t>
+          <t>Toán
+Giáo viên CN 14</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -4810,14 +4810,14 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Đạo đức
-Giáo viên CN 14</t>
+          <t>Thể dục
+Giáo viên TD 2</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 2</t>
+          <t>Công nghệ
+Giáo viên BM 3</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -4888,16 +4888,16 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
+          <t>Đạo đức
+Giáo viên CN 14</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
           <t>Thể dục
 Giáo viên TD 2</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Thể dục
-Giáo viên TD 2</t>
-        </is>
-      </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Nghỉ</t>
@@ -4968,13 +4968,13 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 15</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 15</t>
         </is>
       </c>
@@ -5011,8 +5011,8 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 15</t>
+          <t>Tiếng Anh
+Giáo viên TA 2</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5042,14 +5042,14 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Tin học
-Giáo viên TH 1</t>
+          <t>Tiếng Việt
+Giáo viên CN 15</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 2</t>
+          <t>Tiếng Việt
+Giáo viên CN 15</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -5079,13 +5079,13 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Toán
-Giáo viên CN 15</t>
+          <t>Tiếng Anh
+Giáo viên TA 2</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 15</t>
         </is>
       </c>
@@ -5120,14 +5120,14 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 2</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
           <t>Toán tăng cường
 Giáo viên CN 15</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Tin học
+Giáo viên TH 1</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -5156,14 +5156,14 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
           <t>Thể dục
 Giáo viên TD 2</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -5192,16 +5192,16 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
+          <t>TNXH
+Giáo viên BM 3</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
           <t>Đạo đức
 Giáo viên CN 15</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>TNXH
-Giáo viên BM 3</t>
-        </is>
-      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
           <t>HĐTN
@@ -5284,7 +5284,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 16</t>
         </is>
       </c>
@@ -5309,8 +5309,8 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 2</t>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -5321,8 +5321,8 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 16</t>
+          <t>Công nghệ
+Giáo viên BM 4</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -5346,20 +5346,20 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
           <t>Tiếng Anh
 Giáo viên TA 2</t>
         </is>
       </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Anh
+Giáo viên TA 2</t>
+        </is>
+      </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 2</t>
+          <t>Tiếng Việt
+Giáo viên CN 16</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 16</t>
         </is>
       </c>
@@ -5430,14 +5430,14 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Tin học
-Giáo viên TH 1</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
           <t>TNXH
 Giáo viên BM 4</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Anh
+Giáo viên TA 2</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -5472,8 +5472,8 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 2</t>
+          <t>Tin học
+Giáo viên TH 1</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -5496,8 +5496,8 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Công nghệ
-Giáo viên BM 4</t>
+          <t>Thể dục
+Giáo viên TD 2</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -5588,7 +5588,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 17</t>
         </is>
       </c>
@@ -5600,7 +5600,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 17</t>
         </is>
       </c>
@@ -5631,13 +5631,13 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 2</t>
+          <t>Tiếng Việt
+Giáo viên CN 17</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>TV tăng cường
 Giáo viên CN 17</t>
         </is>
       </c>
@@ -5662,19 +5662,19 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
           <t>Tiếng Việt
 Giáo viên CN 17</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Tin học
-Giáo viên TH 1</t>
-        </is>
-      </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 17</t>
         </is>
       </c>
@@ -5699,14 +5699,14 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
+          <t>Toán
+Giáo viên CN 17</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>TNXH
-Giáo viên BM 4</t>
+          <t>Tin học
+Giáo viên TH 1</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -5740,13 +5740,13 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
           <t>Toán tăng cường
-Giáo viên CN 17</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
 Giáo viên CN 17</t>
         </is>
       </c>
@@ -5782,8 +5782,8 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>TV tăng cường
-Giáo viên CN 17</t>
+          <t>Tiếng Anh
+Giáo viên TA 2</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -5806,22 +5806,22 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
+          <t>TNXH
+Giáo viên BM 4</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Đạo đức
+Giáo viên CN 17</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
           <t>Thể dục
 Giáo viên TD 2</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>Đạo đức
-Giáo viên CN 17</t>
-        </is>
-      </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
           <t>HĐTN
@@ -5898,7 +5898,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 18</t>
         </is>
       </c>
@@ -5929,8 +5929,8 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 3</t>
+          <t>Tin học
+Giáo viên TH 1</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -5966,16 +5966,16 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
+          <t>Toán
+Giáo viên CN 18</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
           <t>Thể dục
 Giáo viên TD 2</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 18</t>
-        </is>
-      </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Tiếng Anh
@@ -5984,7 +5984,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>TNXH
+          <t>Công nghệ
 Giáo viên BM 4</t>
         </is>
       </c>
@@ -6003,20 +6003,20 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
+          <t>Tiếng Anh
+Giáo viên TA 3</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
           <t>Toán
 Giáo viên CN 18</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
-        </is>
-      </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Tin học
-Giáo viên TH 1</t>
+          <t>Toán
+Giáo viên CN 18</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -6050,14 +6050,14 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
+          <t>Tiếng Anh
+Giáo viên TA 2</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
           <t>Thể dục
 Giáo viên TD 2</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>Toán
-Giáo viên CN 18</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -6086,19 +6086,19 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 2</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
           <t>Toán tăng cường
 Giáo viên CN 18</t>
         </is>
       </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
+        </is>
+      </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Công nghệ
+          <t>TNXH
 Giáo viên BM 4</t>
         </is>
       </c>
@@ -6122,14 +6122,14 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
+          <t>TNXH
+Giáo viên BM 4</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
           <t>HĐTN
 Giáo viên CN 18</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>TNXH
-Giáo viên BM 4</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -6296,20 +6296,20 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>Thể dục
+Giáo viên TD 2</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>Tiếng Anh
 Giáo viên TA 3</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Anh
-Giáo viên TA 3</t>
-        </is>
-      </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 2</t>
+          <t>Toán
+Giáo viên CN 19</t>
         </is>
       </c>
     </row>
@@ -6321,32 +6321,32 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Thể dục
+Giáo viên TD 2</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Toán
 Giáo viên CN 19</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
+Giáo viên CN 19</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Mỹ thuật
 Giáo viên MT 1</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 19</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Toán
-Giáo viên CN 19</t>
         </is>
       </c>
     </row>
@@ -6358,14 +6358,14 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>Tiếng Việt
+Giáo viên CN 19</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>Tiếng Anh
 Giáo viên TA 3</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Toán
-Giáo viên CN 19</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -6399,20 +6399,20 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 2</t>
+          <t>Kỹ năng sống
+Giáo viên QL 1</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Anh
-Giáo viên TA 3</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Tin học
 Giáo viên TH 1</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Khoa học
+Giáo viên CN 19</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -6435,20 +6435,20 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>Tiếng Anh
+Giáo viên TA 3</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
           <t>Toán tăng cường
 Giáo viên CN 19</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Khoa học
-Giáo viên CN 19</t>
-        </is>
-      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Kỹ năng sống
-Giáo viên QL 1</t>
+          <t>Tiếng Anh
+Giáo viên TA 3</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -6477,16 +6477,16 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>Đạo đức
+Giáo viên CN 19</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>Công nghệ
 Giáo viên BM 4</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Đạo đức
-Giáo viên CN 19</t>
-        </is>
-      </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>HĐTN
@@ -6563,7 +6563,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 20</t>
         </is>
       </c>
@@ -6581,7 +6581,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 20</t>
         </is>
       </c>
@@ -6594,20 +6594,20 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 2</t>
+          <t>Toán
+Giáo viên CN 20</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Công nghệ
-Giáo viên BM 4</t>
+          <t>Tiếng Việt
+Giáo viên CN 20</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
+          <t>Tiếng Việt
+Giáo viên CN 20</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -6618,8 +6618,8 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Toán
-Giáo viên CN 20</t>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
         </is>
       </c>
     </row>
@@ -6631,32 +6631,32 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Anh
+Giáo viên TA 3</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Công nghệ
+Giáo viên BM 4</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Thể dục
+Giáo viên TD 2</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
 Giáo viên CN 20</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Tiếng Việt
 Giáo viên CN 20</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 20</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 20</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
         </is>
       </c>
     </row>
@@ -6674,14 +6674,14 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
+          <t>Toán
+Giáo viên CN 20</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>Tiếng Anh
 Giáo viên TA 3</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 20</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -6709,20 +6709,20 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Toán tăng cường
-Giáo viên CN 20</t>
+          <t>Thể dục
+Giáo viên TD 2</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Lịch sử - Địa lý
-Giáo viên CN 20</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Tiếng Anh
 Giáo viên TA 3</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Khoa học
+Giáo viên CN 20</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -6745,20 +6745,20 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 3</t>
+          <t>Toán tăng cường
+Giáo viên CN 20</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Khoa học
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Lịch sử - Địa lý
 Giáo viên CN 20</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Thể dục
-Giáo viên TD 2</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -6781,22 +6781,22 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>Lịch sử - Địa lý
+Giáo viên CN 20</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>HĐTN
+Giáo viên CN 20</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>Đạo đức
 Giáo viên CN 20</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>HĐTN
-Giáo viên CN 20</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Lịch sử - Địa lý
-Giáo viên CN 20</t>
-        </is>
-      </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Kỹ năng sống
@@ -6891,7 +6891,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 21</t>
         </is>
       </c>
@@ -6904,16 +6904,16 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Toán
-Giáo viên CN 21</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
           <t>Tiếng Anh
 Giáo viên TA 3</t>
         </is>
       </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Thể dục
+Giáo viên TD 2</t>
+        </is>
+      </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Tin học
@@ -6928,8 +6928,8 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Mỹ thuật
-Giáo viên MT 1</t>
+          <t>Tiếng Anh
+Giáo viên TA 3</t>
         </is>
       </c>
     </row>
@@ -6941,31 +6941,31 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 3</t>
+          <t>Toán
+Giáo viên CN 21</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 2</t>
+          <t>Tiếng Việt
+Giáo viên CN 21</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
+          <t>Mỹ thuật
+Giáo viên MT 1</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
           <t>Tiếng Việt
 Giáo viên CN 21</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 21</t>
-        </is>
-      </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 21</t>
         </is>
       </c>
@@ -7019,19 +7019,19 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
+          <t>Toán tăng cường
+Giáo viên CN 21</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
           <t>Khoa học
 Giáo viên CN 21</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Lịch sử - Địa lý
-Giáo viên CN 21</t>
-        </is>
-      </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Toán tăng cường
+          <t>Khoa học
 Giáo viên CN 21</t>
         </is>
       </c>
@@ -7061,20 +7061,20 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Khoa học
-Giáo viên CN 21</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
           <t>Tiếng Anh
 Giáo viên TA 3</t>
         </is>
       </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Lịch sử - Địa lý
+Giáo viên CN 21</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
+          <t>Lịch sử - Địa lý
+Giáo viên CN 21</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -7091,26 +7091,26 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
+          <t>Đạo đức
+Giáo viên CN 21</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
           <t>Kỹ năng sống
 Giáo viên QL 1</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>HĐTN
 Giáo viên CN 21</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Đạo đức
-Giáo viên CN 21</t>
-        </is>
-      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Lịch sử - Địa lý
-Giáo viên CN 21</t>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -7214,20 +7214,20 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
+          <t>Tiếng Việt
+Giáo viên CN 22</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
           <t>Mỹ thuật
 Giáo viên MT 1</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Thể dục
-Giáo viên TD 2</t>
-        </is>
-      </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 22</t>
+          <t>Tiếng Anh
+Giáo viên TA 3</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -7251,7 +7251,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 22</t>
         </is>
       </c>
@@ -7288,20 +7288,20 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
 Giáo viên CN 22</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Tiếng Việt
 Giáo viên CN 22</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Anh
-Giáo viên TA 3</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -7341,8 +7341,8 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
+          <t>Công nghệ
+Giáo viên BM 4</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -7365,20 +7365,20 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Công nghệ
-Giáo viên BM 4</t>
+          <t>Tin học
+Giáo viên TH 1</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Thể dục
+Giáo viên TD 2</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>Khoa học
 Giáo viên CN 22</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Tin học
-Giáo viên TH 1</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -7407,16 +7407,16 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
+          <t>Lịch sử - Địa lý
+Giáo viên CN 22</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
           <t>Kỹ năng sống
 Giáo viên QL 1</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Lịch sử - Địa lý
-Giáo viên CN 22</t>
-        </is>
-      </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
           <t>HĐTN
@@ -7493,13 +7493,13 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 23</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 23</t>
         </is>
       </c>
@@ -7530,26 +7530,26 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
+          <t>Tiếng Anh
+Giáo viên TA 3</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
           <t>Tiếng Việt
 Giáo viên CN 23</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
+Giáo viên CN 23</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>Thể dục
 Giáo viên TD 2</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 23</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Anh
-Giáo viên TA 3</t>
         </is>
       </c>
     </row>
@@ -7561,20 +7561,20 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Kỹ năng sống
-Giáo viên BM 4</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Toán
-Giáo viên CN 23</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
           <t>Mỹ thuật
 Giáo viên MT 1</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
+Giáo viên CN 23</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Tin học
+Giáo viên TH 1</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -7604,13 +7604,13 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Tin học
-Giáo viên TH 1</t>
+          <t>Âm nhạc
+Giáo viên ÂN 1</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 23</t>
         </is>
       </c>
@@ -7639,20 +7639,20 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
+          <t>Toán tăng cường
+Giáo viên CN 23</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
           <t>Khoa học
 Giáo viên CN 23</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Âm nhạc
-Giáo viên ÂN 1</t>
-        </is>
-      </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Lịch sử - Địa lý
-Giáo viên CN 23</t>
+          <t>Tiếng Anh
+Giáo viên TA 3</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -7675,20 +7675,20 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Toán tăng cường
-Giáo viên CN 23</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Anh
-Giáo viên TA 3</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
           <t>Khoa học
 Giáo viên CN 23</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Lịch sử - Địa lý
+Giáo viên CN 23</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Kỹ năng sống
+Giáo viên BM 4</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -7717,16 +7717,16 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
+          <t>HĐTN
+Giáo viên CN 23</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
           <t>Lịch sử - Địa lý
 Giáo viên CN 23</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>HĐTN
-Giáo viên CN 23</t>
-        </is>
-      </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
           <t>Công nghệ
@@ -7803,13 +7803,13 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 24</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 24</t>
         </is>
       </c>
@@ -7834,25 +7834,25 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 24</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
+          <t>Công nghệ
+Giáo viên BM 4</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
           <t>Tiếng Việt
 Giáo viên CN 24</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Anh
-Giáo viên TA 4</t>
-        </is>
-      </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Mỹ thuật
+          <t>Âm nhạc
 Giáo viên BM 5</t>
         </is>
       </c>
@@ -7871,8 +7871,8 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Tin học
-Giáo viên TH 1</t>
+          <t>Tiếng Việt
+Giáo viên CN 24</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -7883,8 +7883,8 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 24</t>
+          <t>Tiếng Anh
+Giáo viên TA 4</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -7908,19 +7908,19 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Anh
+Giáo viên TA 4</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
 Giáo viên CN 24</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>Toán
-Giáo viên CN 24</t>
-        </is>
-      </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Toán tăng cường
+          <t>Toán
 Giáo viên CN 24</t>
         </is>
       </c>
@@ -7949,19 +7949,19 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Kỹ năng sống
-Giáo viên BM 4</t>
+          <t>Tin học
+Giáo viên TH 1</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Công nghệ
-Giáo viên BM 4</t>
+          <t>Khoa học
+Giáo viên CN 24</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Khoa học
+          <t>Toán tăng cường
 Giáo viên CN 24</t>
         </is>
       </c>
@@ -7985,20 +7985,20 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 4</t>
+          <t>Kỹ năng sống
+Giáo viên BM 4</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Lịch sử - Địa lý
+Giáo viên CN 24</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>Thể dục
 Giáo viên TD 3</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>Đạo đức
-Giáo viên CN 24</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -8033,13 +8033,13 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Lịch sử - Địa lý
+          <t>Đạo đức
 Giáo viên CN 24</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
+          <t>Mỹ thuật
 Giáo viên BM 5</t>
         </is>
       </c>
@@ -8164,7 +8164,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 25</t>
         </is>
       </c>
@@ -8189,20 +8189,20 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 25</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>Tiếng Anh
 Giáo viên TA 4</t>
         </is>
       </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Mỹ thuật
+Giáo viên BM 5</t>
+        </is>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 25</t>
+          <t>Thể dục
+Giáo viên TD 3</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -8213,8 +8213,8 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Công nghệ
-Giáo viên BM 4</t>
+          <t>Toán
+Giáo viên CN 25</t>
         </is>
       </c>
     </row>
@@ -8238,20 +8238,20 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Kỹ năng sống
+          <t>Tiếng Việt
+Giáo viên CN 25</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
+Giáo viên CN 25</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Công nghệ
 Giáo viên BM 4</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 25</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Toán
-Giáo viên CN 25</t>
         </is>
       </c>
     </row>
@@ -8263,8 +8263,8 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 4</t>
+          <t>Tiếng Việt
+Giáo viên CN 25</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -8275,7 +8275,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 25</t>
         </is>
       </c>
@@ -8304,8 +8304,8 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên BM 5</t>
+          <t>Kỹ năng sống
+Giáo viên BM 4</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -8316,8 +8316,8 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 3</t>
+          <t>Toán tăng cường
+Giáo viên CN 25</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -8346,8 +8346,8 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Toán tăng cường
-Giáo viên CN 25</t>
+          <t>Tiếng Anh
+Giáo viên TA 4</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -8382,7 +8382,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Mỹ thuật
+          <t>Âm nhạc
 Giáo viên BM 5</t>
         </is>
       </c>
@@ -8499,14 +8499,14 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 3</t>
+          <t>Tiếng Việt
+Giáo viên CN 26</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 26</t>
+          <t>Tiếng Anh
+Giáo viên TA 4</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -8548,20 +8548,20 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 4</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Việt
-Giáo viên CN 26</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
           <t>Công nghệ
 Giáo viên BM 4</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
+Giáo viên CN 26</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Thể dục
+Giáo viên TD 3</t>
         </is>
       </c>
     </row>
@@ -8573,14 +8573,14 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
+          <t>Kỹ năng sống
+Giáo viên BM 4</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
           <t>Tiếng Việt
 Giáo viên CN 26</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Tiếng Anh
-Giáo viên TA 4</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -8614,20 +8614,20 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
+          <t>Mỹ thuật
+Giáo viên BM 5</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Khoa học
+Giáo viên CN 26</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>Tiếng Anh
 Giáo viên TA 4</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Khoa học
-Giáo viên CN 26</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Lịch sử - Địa lý
-Giáo viên CN 26</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -8650,20 +8650,20 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
+          <t>Tiếng Anh
+Giáo viên TA 4</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Lịch sử - Địa lý
+Giáo viên CN 26</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
           <t>Khoa học
 Giáo viên CN 26</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Lịch sử - Địa lý
-Giáo viên CN 26</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Kỹ năng sống
-Giáo viên BM 4</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -8686,22 +8686,22 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>Lịch sử - Địa lý
+Giáo viên CN 26</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Đạo đức
+Giáo viên CN 26</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>Âm nhạc
 Giáo viên BM 5</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Đạo đức
-Giáo viên CN 26</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Mỹ thuật
-Giáo viên BM 5</t>
-        </is>
-      </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>HĐTN
@@ -8778,7 +8778,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 27</t>
         </is>
       </c>
@@ -8796,7 +8796,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
+          <t>Toán
 Giáo viên CN 27</t>
         </is>
       </c>
@@ -8809,32 +8809,32 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Công nghệ
-Giáo viên BM 4</t>
+          <t>Toán
+Giáo viên CN 27</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
+          <t>Tin học
+Giáo viên TH 1</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
           <t>Tiếng Việt
 Giáo viên CN 27</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>Thể dục
 Giáo viên TD 3</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>Thể dục
-Giáo viên TD 3</t>
-        </is>
-      </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Toán
-Giáo viên CN 27</t>
+          <t>Kỹ năng sống
+Giáo viên BM 4</t>
         </is>
       </c>
     </row>
@@ -8846,14 +8846,14 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Công nghệ
+Giáo viên BM 4</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
 Giáo viên CN 27</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Kỹ năng sống
-Giáo viên BM 4</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -8870,8 +8870,8 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 4</t>
+          <t>Tiếng Việt
+Giáo viên CN 27</t>
         </is>
       </c>
     </row>
@@ -8889,14 +8889,14 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 27</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 27</t>
+          <t>Tiếng Anh
+Giáo viên TA 4</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -8924,8 +8924,8 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Tin học
-Giáo viên TH 1</t>
+          <t>Khoa học
+Giáo viên CN 27</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -8936,8 +8936,8 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Âm nhạc
-Giáo viên BM 5</t>
+          <t>Thể dục
+Giáo viên TD 3</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -8960,20 +8960,20 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Khoa học
+          <t>Toán tăng cường
 Giáo viên CN 27</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Âm nhạc
+Giáo viên BM 5</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Mỹ thuật
 Giáo viên BM 5</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Toán tăng cường
-Giáo viên CN 27</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -9002,22 +9002,22 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
+          <t>Lịch sử - Địa lý
+Giáo viên CN 27</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
           <t>HĐTN
 Giáo viên CN 27</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Lịch sử - Địa lý
 Giáo viên CN 27</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>Lịch sử - Địa lý
-Giáo viên CN 27</t>
-        </is>
-      </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Nghỉ</t>
@@ -9088,7 +9088,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 28</t>
         </is>
       </c>
@@ -9106,7 +9106,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Khoa học
+          <t>Toán
 Giáo viên CN 28</t>
         </is>
       </c>
@@ -9119,8 +9119,8 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 4</t>
+          <t>Thể dục
+Giáo viên TD 3</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -9143,7 +9143,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Toán
+          <t>Tiếng Việt
 Giáo viên CN 28</t>
         </is>
       </c>
@@ -9162,8 +9162,8 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 28</t>
+          <t>Tiếng Anh
+Giáo viên TA 4</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -9180,8 +9180,8 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 28</t>
+          <t>Tiếng Anh
+Giáo viên TA 4</t>
         </is>
       </c>
     </row>
@@ -9199,8 +9199,8 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Thể dục
-Giáo viên TD 3</t>
+          <t>Toán
+Giáo viên CN 28</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -9234,8 +9234,8 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Toán tăng cường
-Giáo viên CN 28</t>
+          <t>Tiếng Anh
+Giáo viên TA 4</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -9246,8 +9246,8 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 4</t>
+          <t>Khoa học
+Giáo viên CN 28</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -9276,14 +9276,14 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 4</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
           <t>Thể dục
 Giáo viên TD 3</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Toán tăng cường
+Giáo viên CN 28</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -9312,13 +9312,13 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
+          <t>Lịch sử - Địa lý
+Giáo viên CN 28</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
           <t>HĐTN
-Giáo viên CN 28</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Lịch sử - Địa lý
 Giáo viên CN 28</t>
         </is>
       </c>
@@ -9429,20 +9429,20 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Kỹ năng sống
+          <t>Công nghệ
 Giáo viên BM 5</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Mỹ thuật
-Giáo viên BM 5</t>
+          <t>Tiếng Việt
+Giáo viên CN 29</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 29</t>
+          <t>Tiếng Anh
+Giáo viên TA 4</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -9472,8 +9472,8 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Anh
-Giáo viên TA 4</t>
+          <t>Tin học
+Giáo viên TH 1</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -9509,14 +9509,14 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-Giáo viên CN 29</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
           <t>Tiếng Anh
 Giáo viên TA 4</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt
+Giáo viên CN 29</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -9556,8 +9556,8 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Khoa học
-Giáo viên CN 29</t>
+          <t>Mỹ thuật
+Giáo viên BM 5</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -9580,20 +9580,20 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Tin học
-Giáo viên TH 1</t>
+          <t>Lịch sử - Địa lý
+Giáo viên CN 29</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Đạo đức
+          <t>Lịch sử - Địa lý
 Giáo viên CN 29</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Công nghệ
-Giáo viên BM 5</t>
+          <t>Khoa học
+Giáo viên CN 29</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -9616,19 +9616,19 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Lịch sử - Địa lý
+          <t>Kỹ năng sống
+Giáo viên BM 5</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Đạo đức
 Giáo viên CN 29</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>HĐTN
-Giáo viên CN 29</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>Lịch sử - Địa lý
 Giáo viên CN 29</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Output templates with plain class names and overtime/spare columns
Regenerated with tools/mau_dau_ra.py from the fake-name school (code
428A-3655-C110, unchanged).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B1DqxLw2MywB8g5N8E14F5
</commit_message>
<xml_diff>
--- a/data/Output_Template_TKB_V8.xlsx
+++ b/data/Output_Template_TKB_V8.xlsx
@@ -464,7 +464,7 @@
   <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.5" customWidth="1" min="1" max="1"/>
+    <col width="5.7" customWidth="1" min="1" max="1"/>
     <col width="12.1" customWidth="1" min="2" max="2"/>
     <col width="10.9" customWidth="1" min="3" max="3"/>
     <col width="21.5" customWidth="1" min="4" max="4"/>
@@ -519,7 +519,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>LỚP 1/1</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -829,7 +829,7 @@
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>LỚP 1/2</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -1139,7 +1139,7 @@
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>LỚP 1/3</t>
+          <t>1/3</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1449,7 +1449,7 @@
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>LỚP 1/4</t>
+          <t>1/4</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1759,7 +1759,7 @@
     <row r="42" ht="42" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>LỚP 1/5</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -2069,7 +2069,7 @@
     <row r="52" ht="42" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>LỚP 1/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -2369,7 +2369,7 @@
   <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.5" customWidth="1" min="1" max="1"/>
+    <col width="5.7" customWidth="1" min="1" max="1"/>
     <col width="12.1" customWidth="1" min="2" max="2"/>
     <col width="10.9" customWidth="1" min="3" max="3"/>
     <col width="21.5" customWidth="1" min="4" max="4"/>
@@ -2424,7 +2424,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>LỚP 2/1</t>
+          <t>2/1</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -2734,7 +2734,7 @@
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>LỚP 2/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -3044,7 +3044,7 @@
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>LỚP 2/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -3354,7 +3354,7 @@
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>LỚP 2/4</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -3664,7 +3664,7 @@
     <row r="42" ht="42" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>LỚP 2/5</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -3974,7 +3974,7 @@
     <row r="52" ht="42" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>LỚP 2/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -4274,7 +4274,7 @@
   <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.5" customWidth="1" min="1" max="1"/>
+    <col width="5.7" customWidth="1" min="1" max="1"/>
     <col width="12.1" customWidth="1" min="2" max="2"/>
     <col width="10.9" customWidth="1" min="3" max="3"/>
     <col width="21.5" customWidth="1" min="4" max="4"/>
@@ -4329,7 +4329,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>LỚP 3/1</t>
+          <t>3/1</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -4639,7 +4639,7 @@
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>LỚP 3/2</t>
+          <t>3/2</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -4949,7 +4949,7 @@
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>LỚP 3/3</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -5259,7 +5259,7 @@
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>LỚP 3/4</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -5569,7 +5569,7 @@
     <row r="42" ht="42" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>LỚP 3/5</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -5879,7 +5879,7 @@
     <row r="52" ht="42" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>LỚP 3/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -6179,7 +6179,7 @@
   <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.5" customWidth="1" min="1" max="1"/>
+    <col width="5.7" customWidth="1" min="1" max="1"/>
     <col width="12.1" customWidth="1" min="2" max="2"/>
     <col width="10.9" customWidth="1" min="3" max="3"/>
     <col width="21.5" customWidth="1" min="4" max="4"/>
@@ -6234,7 +6234,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>LỚP 4/1</t>
+          <t>4/1</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -6544,7 +6544,7 @@
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>LỚP 4/2</t>
+          <t>4/2</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -6854,7 +6854,7 @@
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>LỚP 4/3</t>
+          <t>4/3</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -7164,7 +7164,7 @@
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>LỚP 4/4</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -7474,7 +7474,7 @@
     <row r="42" ht="42" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>LỚP 4/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -7784,7 +7784,7 @@
     <row r="52" ht="42" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>LỚP 4/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -8084,7 +8084,7 @@
   <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.5" customWidth="1" min="1" max="1"/>
+    <col width="5.7" customWidth="1" min="1" max="1"/>
     <col width="12.1" customWidth="1" min="2" max="2"/>
     <col width="10.9" customWidth="1" min="3" max="3"/>
     <col width="21.5" customWidth="1" min="4" max="4"/>
@@ -8139,7 +8139,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>LỚP 5/1</t>
+          <t>5/1</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -8449,7 +8449,7 @@
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>LỚP 5/2</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -8759,7 +8759,7 @@
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>LỚP 5/3</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -9069,7 +9069,7 @@
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>LỚP 5/4</t>
+          <t>5/4</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -9379,7 +9379,7 @@
     <row r="42" ht="42" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>LỚP 5/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">

</xml_diff>